<commit_message>
Complete lesson 21: Refactored scraper into modular functions
</commit_message>
<xml_diff>
--- a/all_pages_quotes_styled.xlsx
+++ b/all_pages_quotes_styled.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ဟယ်ရီ၊ ငါတို့ရဲ့ အရည်အချင်းတွေထက် ငါတို့အမှန်တကယ်ရှိတာကို ပြသတဲ့ ငါတို့ရဲ့ ရွေးချယ်မှုပဲ။</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>အောင်မြင်သူတစ်ယောက်ဖြစ်ဖို့ မကြိုးစားပါနဲ့။ တန်ဖိုးထားတတ်သူဖြစ်ပါစေ။</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ငါမအောင်မြင်ဘူး။ အလုပ်မဖြစ်နိုင်တဲ့ နည်းလမ်း 10,000 လောက်ကို ရှာတွေ့ခဲ့ပါတယ်။</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>နေရောင်ခြည်မရှိသောနေ့သည် ညနှင့်တူသည်။</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>ဒီဘဝက မင်းလုပ်ထားတာ။ ဘာပဲဖြစ်ဖြစ် တခါတရံ စိတ်ရှုပ်သွားတတ်ပါတယ်၊ ဒါဟာ စကြာဝဠာအမှန်တရားပါ။ ဒါပေမယ့် ကောင်းတဲ့ အပိုင်းကတော့ ဘယ်လို ရှုပ်အောင် လုပ်မယ်ဆိုတာကို သင် ဆုံးဖြတ်ရလိမ့်မယ်။ ကောင်မလေးတွေက မင်းရဲ့သူငယ်ချင်းတွေဖြစ်လိမ့်မယ်၊ ဘာပဲဖြစ်ဖြစ် သူတို့ဒီလိုလုပ်လိမ့်မယ်။ ဒါပေမယ့် တစ်ချို့က လာကြတယ်၊ တစ်ချို့က သွားကြတာကို သတိရပါ။ အရာရာတိုင်းမှာ မင်းနဲ့အတူရှိနေသူတွေ - သူတို့က မင်းရဲ့အကောင်းဆုံးသူငယ်ချင်းတွေပါ။ သူတို့ကို လက်မလွှတ်လိုက်ပါနဲ့။ ညီမလေးတွေက ကမ္ဘာပေါ်မှာ အကောင်းဆုံးသူငယ်ချင်းတွေဖြစ်တယ်ဆိုတာ သတိရပါ။ ချစ်သူတွေဆိုလည်း လာလည်ကြမယ်နော်။ ကလေး၊ ငါပြောတာကိုမုန်းတယ်၊ အများစုဟာ - တကယ်တော့ သူတို့အားလုံးက မင်းရဲ့စိတ်နှလုံးကို ကြေကွဲသွားစေလိမ့်မယ်၊ ဒါပေမယ့် မင်းအရှုံးမပေးဘူးဆိုရင် မင်းရဲ့ချစ်သူကို မင်းဘယ်တော့မှ ရှာတွေ့မှာမဟုတ်ဘူး။ မင်းကိုကျန်းမာစေပြီး အရာအားလုံးအတွက်ဖြစ်စေမယ့် အဲဒီတစ်ဝက်ကို မင်းဘယ်တော့မှ ရှာတွေ့မှာမဟုတ်ဘူး။ တစ်ကြိမ်ကျရှုံးရုံနဲ့ အရာအားလုံး ကျရှုံးမယ်လို့ မဆိုလိုပါဘူး။ ကြိုးစားပါ၊ ကိုင်ပါ၊ အမြဲတမ်း၊ အမြဲတမ်း ကိုယ့်ကိုကိုယ် အမြဲယုံကြည်နေမှာမို့လို့ မင်းမှမဟုတ်ရင် ဘယ်သူကဖြစ်မှာလဲ။ ဒါကြောင့် ခေါင်းကို မြင့်မြင့်ထားပါ၊ မေးစေ့ကို မတ်မတ်ထားပါ၊ အရေးကြီးဆုံးကတော့ ဘဝဟာ လှပပြီး ပြုံးစရာတွေ အများကြီးရှိတာကြောင့် ပြုံးနေလိုက်ပါ။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ချစ်ခြင်းမေတ္တာ ကင်းမဲ့ခြင်း မဟုတ်ဘဲ ခင်မင်ရင်းနှီးမှု ကင်းမဲ့ခြင်းကြောင့် သာယာသော အိမ်ထောင်ရေးကို ဖြစ်စေသည်။</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>လူတွေကို အကဲဖြတ်ရင် သူတို့ကို ချစ်ဖို့ အချိန်မရှိဘူး။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>အလှတရားသည် ကြည့်ရှုသူ၏မျက်လုံးထဲတွင်ရှိပြီး မိုက်မဲသော သို့မဟုတ် အသိမှားမြင်သူအား မျက်ကွင်းညိုစေရန် အခါအားလျော်စွာ လိုအပ်ပေမည်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>သားသမီးတွေကို ဉာဏ်ရည်ထက်မြက်စေချင်ရင် ဒဏ္ဍာရီပုံပြင်တွေကို ဖတ်ပါ။ သူတို့ကို ပိုဉာဏ်ကောင်းစေချင်ရင် ဒဏ္ဍာရီပုံပြင်တွေကို ပိုဖတ်ပါ။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>တစ်ခုခုကို မပျက်ကွက်ဘဲနဲ့ အသက်ရှင်ဖို့ဆိုတာ မဖြစ်နိုင်ပါဘူး၊ သင်အရမ်းသတိကြီးစွာနဲ့ အသက်ရှင်မနေဘူးဆိုရင် သင်ဟာ လုံးဝအသက်မရှင်နိုင်ပါဘူး - ဒီလိုအခြေအနေမျိုးမှာ သင်ဟာ ပုံသေအတိုင်း ကျရှုံးသွားနိုင်ပါတယ်။</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>စာများများဖတ်လေ၊ သိလာလေလေပါပဲ။ များများလေ့လာလေ၊ သွားရမယ့်နေရာတွေ ပိုများလာမယ်။</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>အမှန်တရားကတော့ လူတိုင်းက မင်းကို နာကျင်စေလိမ့်မယ်။ ဒုက္ခရောက်ရကျိုးနပ်တဲ့ သူတွေကိုပဲ ရှာရမယ်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ငါတို့တစ်ယောက်ထဲမဟုတ်ဘူးဆိုတာ သိအောင်ဖတ်တယ်။</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>စာဖတ်သူသည် မသေဆုံးမီ ဘဝပေါင်း တစ်ထောင်ကျော် အသက်ရှင်သည်ဟု Jojen က ဆိုသည်။ မဖတ်ဖူးသောလူသည် တစ်ဦးတည်းသာ အသက်ရှင်သည်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>သင်သည် မုသားကို ယုံကြည်သောကြောင့် နောက်ဆုံးတွင် သင်ကိုယ်တိုင်မှတပါး အခြားမည်သူ့ကိုမျှ ယုံကြည်ရန် သင်ယူပါ။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>မိန်းမကို ရယ်အောင်လုပ်နိုင်ရင် သူ့ကို ဘာမဆိုလုပ်ပေးနိုင်တယ်။</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>အချစ်သည် ကျွန်ုပ်တို့ထင်ထားသည့်အတိုင်း အစပြု၍အဆုံးသတ်မည်မဟုတ်ပေ။ အချစ်သည်စစ်ပွဲတစ်ခုဖြစ်သည်။ အချစ်သည်စစ်ပွဲတစ်ခုဖြစ်သည်။ အချစ်သည် ကြီးပြင်းလာသည်။</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>ငါက ကောင်းပေမယ့် နတ်သမီးမဟုတ်ဘူး။ ငါသည် ဒုစရိုက်ကိုပြုသော်လည်း၊ ငါသည် မာရ်နတ်မဟုတ်၊ ငါဟာ ကမ္ဘာကြီးမှာ ချစ်ဖို့ကြိုးစားနေတဲ့ မိန်းကလေးတစ်ယောက်ပါ။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ကျွန်တော်သာ ရူပဗေဒပညာရှင်မဟုတ်ပါက ဂီတပညာရှင်တစ်ယောက်ဖြစ်နိုင်သည်။ သီချင်းထဲမှာ တွေးတတ်တယ်။ ဂီတထဲမှာ ငါရဲ့ နေ့ခင်းအိပ်မက်တွေကို ရှင်သန်နေတယ်။ ဂီတနဲ့ပတ်သက်ရင် ကျွန်တော့်ဘဝကို မြင်တယ်။</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>မင်းရဲ့နောက်ဆုံးမျှော်လင့်ချက်ဖြစ်ခဲ့တဲ့လူရဲ့မျက်နှာကို မင်းမမေ့ပါနဲ့။</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>နေ့ရက်တိုင်းကို ပြီးအောင်လုပ်ပါ။ သင် တတ်နိုင်သလောက် လုပ်ခဲ့ပြီးပြီ။ အချို့သော လွဲမှားမှုများနှင့် အဓိပ္ပါယ်မဲ့မှုများသည် သံသယဝင်လာမည်မှာ သေချာပါသည်။ သူတို့ကို တတ်နိုင်သမျှ မေ့လိုက်ပါ။ မနက်ဖြန်သည် နေ့သစ်ဖြစ်သည်။ မင်းရဲ့ အဓိပ္ပါယ်ဟောင်းတွေနဲ့ ဖုံးကွယ်ထားနိုင်တဲ့ စိတ်တွေ တည်ငြိမ်စွာနဲ့ စတင်ရလိမ့်မယ်။</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ဘယ်ကိုတွေးပြီး ညာဘက်ကိုတွေးပြီး နိမ့်တွေးပြီး မြင့်အောင်တွေးပါ။ အိုး၊ တွေးကြည့်စမ်းပါ တွေးကြည့်လို့ရတယ်။</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>'Classic' - လူတွေက ချီးမွမ်းပြီး မဖတ်ရတဲ့ စာအုပ်။</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ကိုယ်တကယ်ချစ်တဲ့လူ နည်းနည်းပဲရှိတော့ ကောင်းကောင်းထင်တဲ့သူက နည်းနေသေးတယ်။ ကမ္ဘာကြီးကို ပိုမြင်လေလေ၊ အဲဒါကို မကျေနပ်လေလေ၊ နေ့တိုင်း လူသားဇာတ်ကောင်အားလုံးရဲ့ တသမတ်တည်းဖြစ်တဲ့ ငါ့ယုံကြည်ချက်နဲ့ ကုသိုလ် သို့မဟုတ် အာရုံရဲ့အသွင်အပြင်အပေါ် ထားနိုင်တဲ့ အားကိုးမှုအနည်းငယ်ကို နေ့တိုင်း အတည်ပြုပါတယ်။</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>ဘုရားသခင်သည် ကျွန်ုပ်တို့အတွက် အကောင်းဆုံးလုပ်ဆောင်ပေးမည်ကို ကျွန်ုပ်တို့သံသယဖြစ်စရာမလိုပါ။ အကောင်းဆုံးက ဘယ်လောက်အထိ နာကျင်ရမလဲဆိုတာ တွေးတောနေတယ်။</t>
+          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>အမှန်တရား။” Dumbledore သက်ပြင်းချပြီး “ဒါဟာ လှပပြီး ကြောက်စရာကောင်းတဲ့ အရာဖြစ်ပြီး ဒါကြောင့် သတိကြီးကြီးထားပြီး ဆက်ဆံသင့်ပါတယ်။</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>သေရခြင်းသည် အလွန်ကြီးမားသော စွန့်စားမှုတစ်ခု ဖြစ်လိမ့်မည်။</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>ရေးချင်တဲ့ စာအုပ်ကို ရေးရမယ်။ စာအုပ်က လူကြီးတွေအတွက် အရမ်းခက်ခဲမယ် ဆိုရင်တော့ ကလေးတွေအတွက် ရေးပေးလိုက်ပါ။</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>မထိုက်တန်တဲ့သူတွေကို ဘယ်တော့မှ အမှန်အတိုင်း မပြောပါနဲ့။</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Error 500 (Server Error)!!1500.That’s an error.There was an error. Please try again later.That’s all we know.</t>
+          <t>. . . . . . . . . . . . . . . . . . . . . . .</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">

</xml_diff>